<commit_message>
chore: uncommitted changes - clova, vision, experiments
</commit_message>
<xml_diff>
--- a/experiments/v7_output.xlsx
+++ b/experiments/v7_output.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="전체" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="전체데이터" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,17 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
     </font>
     <font>
       <b val="1"/>
@@ -50,9 +54,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -418,1976 +423,1985 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A285"/>
+  <dimension ref="A1:A287"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>등기부등본 파싱 결과 (v7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
           <t>[__header__]</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>고유번호2849-2018-019318</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>[토지]경기도파주시파평면마산리113-2</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>[【표제부】]</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2023년02월20일</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>경기도파주시파평면</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>마산리113-2</t>
+          <t>2023년02월20일</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1소유권이전1997년09월11일 | 199748428 | 소유자이은470810-※※※※※※※</t>
+          <t>경기도파주시파평면</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>(A 1)Al 42567. 매매경기도 BPA)중부면오전리220-1</t>
+          <t>마산리113-2</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>분할로인하여순위제1번등기를경기도</t>
+          <t>1소유권이전1997년09월11일 | 199748428 | 소유자이은470810-※※※※※※※</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>파주시파평면마산리113-1에서이기</t>
+          <t>(A 1)Al 42567. 매매경기도 BPA)중부면오전리220-1</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>접수 _2018년11월27일</t>
+          <t>분할로인하여순위제1번등기를경기도</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>제99956호</t>
+          <t>파주시파평면마산리113-1에서이기</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2소유권이전2018년12월24일 | 2018년07월24일공유자</t>
+          <t>접수 _2018년11월27일</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>제107414호매매지분2분의1</t>
+          <t>제99956호</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>강성원620910-*※*※※※※※※</t>
+          <t>2소유권이전2018년12월24일 | 2018년07월24일공유자</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>경기도파주시문산읍사임당로65-30</t>
+          <t>제107414호매매지분2분의1</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>지분2분의1</t>
+          <t>강성원620910-*※*※※※※※※</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>@ | ee 7](0728-*%※%※%※※※%※※</t>
+          <t>경기도파주시문산읍사임당로65-30</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>매매목록제2018-3005호</t>
+          <t>지분2분의1</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>32020년03월04일지분2분의1</t>
+          <t>'@ | ee 7](0728-*%※%※%※※※%※※</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>제18166호</t>
+          <t>매매목록제2018-3005호</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>기</t>
+          <t>32020년03월04일지분2분의1</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>열람일시 : 2026년03월31일17시25분59초</t>
+          <t>제18166호</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>7](0728-*※※*※※*※*※※</t>
+          <t>기</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>도파주시문산음사임당로65-30</t>
+          <t>열람일시 : 2026년03월31일17시25분59초</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2020년07월08일2020년07월02일</t>
+          <t>7](0728-*※※*※※*※*※※</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>제56432호해제</t>
+          <t>도파주시문산음사임당로65-30</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>6임의경매개시결정</t>
+          <t>2020년07월08일2020년07월02일</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>웨</t>
+          <t>제56432호해제</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2025141129172 | 202541128172 | 채권자 _ 북파주농업협동조힙15636-0000297</t>
+          <t>6임의경매개시결정</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>제6029598호 _ | 의정부지방법원경기도파주시문산읍</t>
+          <t>웨</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>고양지원의</t>
+          <t>2025141129172 | 202541128172 | 채권자 _ 북파주농업협동조힙15636-0000297</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>임의경매개시결</t>
+          <t>제6029598호 _ | 의정부지방법원경기도파주시문산읍</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>정(2025타경647</t>
+          <t>고양지원의</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>[을 _ 구】(Asa</t>
+          <t>임의경매개시결</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>&lt; 전33 | HS</t>
+          <t>정(2025타경647</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>유 AVA</t>
+          <t>[을 _ 구】(Asa</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>열람일시 : 2026403831417시25분59초</t>
+          <t>&lt; 전33 | HS</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>지]경기도파주시파평면마산리113-2</t>
+          <t>유 AVA</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>[토지</t>
+          <t>열람일시 : 2026403831417시25분59초</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>eves]5199 | a4 en</t>
+          <t>지]경기도파주시파평면마산리113-2</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>권리자및기타사항</t>
+          <t>[토지</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>분할로인하여순위제1번부터2번까지능기를</t>
+          <t>eves]5199 | a4 en</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>경기도파주시파평면마산리113-1에서이기</t>
+          <t>권리자및기타사항</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>AF 20184118274</t>
+          <t>분할로인하여순위제1번부터2번까지능기를</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>3 aS ㅋ 42월34웅22249</t>
+          <t>경기도파주시파평면마산리113-1에서이기</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ANOS = 설정계약</t>
+          <t>AF 20184118274</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>그 TCI</t>
+          <t>3 aS ㅋ 42월34웅22249</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>41번근저당권설정등 | 2018년12월24일 | 20184128249</t>
+          <t>ANOS = 설정계약</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>기말소제107416호해지</t>
+          <t>그 TCI</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>52번지상권설정능기 | 32018년12월24일 | 20184128249</t>
+          <t>41번근저당권설정등 | 2018년12월24일 | 20184128249</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>말소제107417호해지</t>
+          <t>기말소제107416호해지</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>6 {abt ㅋ 42월34웅22494 ′</t>
+          <t>52번지상권설정능기 | 32018년12월24일 | 20184128249</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>제3674348호살종계약범 - 위 - 도자곤부</t>
+          <t>말소제107417호해지</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>73번근저당권설정능 ，2024년02월14일 | 20244281448</t>
+          <t>6 {abt ㅋ 42월34웅22494 ′</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>기말소제10276호해지</t>
+          <t>제3674348호살종계약범 - 위 - 도자곤부</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>86번지상권설정능기 | 2024428149 | 20244281448</t>
+          <t>73번근저당권설정능 ，2024년02월14일 | 20244281448</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>순위번호 | 등기목적접수동기원인권리자및기타사항</t>
+          <t>기말소제10276호해지</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>말소제10277호해지</t>
+          <t>86번지상권설정능기 | 2024428149 | 20244281448</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>9근저당권설정2024년02월14일 ， 2024년02월14일채권최고액금221,000,000원</t>
+          <t>순위번호 | 등기목적접수동기원인권리자및기타사항</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>제10278호설정계약 AEX 이순옥</t>
+          <t>말소제10277호해지</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>근저당권자북파주농업협동조합</t>
+          <t>9근저당권설정2024년02월14일 ， 2024년02월14일채권최고액금221,000,000원</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>115636-0000297</t>
+          <t>제10278호설정계약 AEX 이순옥</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>경기도파주시문산읍문향로75</t>
+          <t>근저당권자북파주농업협동조합</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>(파평지점)</t>
+          <t>115636-0000297</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>공동담보목록제2024-225호</t>
+          <t>경기도파주시문산읍문향로75</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>10근저당권설정2024년02월14일2024년02월14일채권최고액금130,000,000원</t>
+          <t>(파평지점)</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>제10279호설정계약 AEX 이순옥</t>
+          <t>공동담보목록제2024-225호</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>〈_꽤 - ㅠ 7} oS Al]2024-2268.</t>
+          <t>10근저당권설정2024년02월14일2024년02월14일채권최고액금130,000,000원</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>11지상권설정2024톨떨촬욜일20241큭′휠_모끓끝</t>
+          <t>제10279호설정계약 AEX 이순옥</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>제10280호 ㅋ Ag 73 APE</t>
+          <t>〈_꽤 - ㅠ 7} oS Al]2024-2268.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2024144849)</t>
+          <t>11지상권설정2024톨떨촬욜일20241큭′휠_모끓끝</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>제29644호</t>
+          <t>제10280호 ㅋ Ag 73 APE</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2024년04월04일</t>
+          <t>2024144849)</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>설정계약</t>
+          <t>제29644호</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>채권최고액금360,000,000원</t>
+          <t>2024년04월04일</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>채무자강성원</t>
+          <t>설정계약</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>서울특별시마포구마포대로4라길30,106농</t>
+          <t>채권최고액금360,000,000원</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>802호(마포농 , 마포쌍용황금아파트)</t>
+          <t>채무자강성원</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
+          <t>서울특별시마포구마포대로4라길30,106농</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>802호(마포농 , 마포쌍용황금아파트)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
           <t>공동담보목록제2024-558호</t>
         </is>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" s="1" t="inlineStr">
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
         <is>
           <t>[【매매목록】]</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>목록번호 」 2018-3005</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>거래가액 | 금300,000,000원</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>예비란</t>
+          <t>목록번호 」 2018-3005</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>일련번호부동산의표시순위번호</t>
+          <t>거래가액 | 금300,000,000원</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>능기원인경정원인</t>
+          <t>예비란</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>1[토지]경기도파주시파평면마산리산44-72018년07월24일</t>
+          <t>일련번호부동산의표시순위번호</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>매매</t>
+          <t>능기원인경정원인</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2[토지]경기도파주시파평면마산리산44-162018년07월24일</t>
+          <t>1[토지]경기도파주시파평면마산리산44-72018년07월24일</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>3[토지]경기도파주시파평면마산리113-12018년07월24일</t>
+          <t>매매</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
+          <t>2[토지]경기도파주시파평면마산리산44-162018년07월24일</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>3[토지]경기도파주시파평면마산리113-12018년07월24일</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
           <t>4[토지]경기도파주시파평면마산리113-222018년07월24일</t>
         </is>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" s="1" t="inlineStr">
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
         <is>
           <t>[【공동담보목록】]</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>ESS | 2023-233</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>일련번호부동산에관한권리의표시관할능기소명</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>4202414281424</t>
+          <t>ESS | 2023-233</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>체30833호제10276호</t>
+          <t>일련번호부동산에관한권리의표시관할능기소명</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>분할로 - 완 ㅎ 해지</t>
+          <t>4202414281424</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2근3 宰 20e 2024년02월14일</t>
+          <t>체30833호제10276호</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>제36833초제10276호</t>
+          <t>분할로 - 완 ㅎ 해지</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>해지</t>
+          <t>2근3 宰 20e 2024년02월14일</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>320241424144</t>
+          <t>제36833초제10276호</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>A 10276</t>
+          <t>해지</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>기타사항</t>
+          <t>320241424144</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>이0</t>
+          <t>A 10276</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>[포</t>
+          <t>기타사항</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>일련번호부동산에</t>
+          <t>이0</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>한권리의</t>
+          <t>[포</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>시</t>
+          <t>일련번호부동산에</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>생성원인변경 / 소멸</t>
+          <t>한권리의</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>파주능분활로 - 완하여 | 해지</t>
+          <t>시</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2024년02월14일</t>
+          <t>생성원인변경 / 소멸</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>제10276호</t>
+          <t>파주능분활로 - 완하여 | 해지</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2023년07월25일</t>
+          <t>2024년02월14일</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>제53675호</t>
+          <t>제10276호</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>HAE 인하여</t>
+          <t>2023년07월25일</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>62024년02월14일</t>
+          <t>제53675호</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>우2024년02월14일</t>
+          <t>HAE 인하여</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>목록번호 」 2024-225쿨</t>
+          <t>62024년02월14일</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>제10278호</t>
+          <t>우2024년02월14일</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>설정계약으로</t>
+          <t>목록번호 」 2024-225쿨</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>인하여</t>
+          <t>제10278호</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>[토지]경기도</t>
+          <t>설정계약으로</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>파주시파평면마산리</t>
+          <t>인하여</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>[토지]경기도파주시파평면마산리 ， 의정부지2024년02월14일</t>
+          <t>[토지]경기도</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>113-2고양지원제10278호</t>
+          <t>파주시파평면마산리</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>파주시파평면마산리 | 의정부지2024년02월14일</t>
+          <t>[토지]경기도파주시파평면마산리 ， 의정부지2024년02월14일</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>고양지원제10278호</t>
+          <t>113-2고양지원제10278호</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>파주능기설정계약으로</t>
+          <t>파주시파평면마산리 | 의정부지2024년02월14일</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>일련번호부동산에관한권리의표시관할등기소명호</t>
+          <t>고양지원제10278호</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>4 | [eA]경기도파주시파평면마산리 | 의정부지방법원 _ | 92024142914)</t>
+          <t>파주능기설정계약으로</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>산44-16고양지원제10278호</t>
+          <t>일련번호부동산에관한권리의표시관할등기소명호</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>파주등기소설정계약으로</t>
+          <t>4 | [eA]경기도파주시파평면마산리 | 의정부지방법원 _ | 92024142914)</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>5 | [토지]경기도파주시파평면마산리 | 의정부지방법원2024142914)</t>
+          <t>산44-16고양지원제10278호</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>113-4고양지원제10278호</t>
+          <t>파주등기소설정계약으로</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>경기도파주시파평면마산리 | 의정부지방법원20241429149)</t>
+          <t>5 | [토지]경기도파주시파평면마산리 | 의정부지방법원2024142914)</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>115-21고양지원제10278호</t>
+          <t>113-4고양지원제10278호</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>경기도파주시파평면마산리20241429149)</t>
+          <t>경기도파주시파평면마산리 | 의정부지방법원20241429149)</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>115-22 Al]102788.</t>
+          <t>115-21고양지원제10278호</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Or 설정계약으로</t>
+          <t>경기도파주시파평면마산리20241429149)</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>6220인하여</t>
+          <t>115-22 Al]102788.</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>경기도파주시파평면마산리 | 의정부지20241429149)</t>
+          <t>Or 설정계약으로</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>115-24고양지원제10278호</t>
+          <t>6220인하여</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>파주등기설정계약으로</t>
+          <t>경기도파주시파평면마산리 | 의정부지20241429149)</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>경기도파주시파평면마산리 | 의정부지방법원2024142914)</t>
+          <t>115-24고양지원제10278호</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>115-20고양지원제10278호</t>
+          <t>파주등기설정계약으로</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>10 | [토지]경기도파주시파평면마산리 | 의정부지방법원2024142914)</t>
+          <t>경기도파주시파평면마산리 | 의정부지방법원2024142914)</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>115-23고양지원제10278호</t>
+          <t>115-20고양지원제10278호</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>11 。 | | [토지]경기도파주시파평면마산리 | 의정부지방법원20241429149)</t>
+          <t>10 | [토지]경기도파주시파평면마산리 | 의정부지방법원2024142914)</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>108-3고양지원제10278호</t>
+          <t>115-23고양지원제10278호</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>구스기소</t>
+          <t>11 。 | | [토지]경기도파주시파평면마산리 | 의정부지방법원20241429149)</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>생성원인</t>
+          <t>108-3고양지원제10278호</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>12[토지]경기도파주시파평면마산리</t>
+          <t>구스기소</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>브</t>
+          <t>생성원인</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>의정부지방범원</t>
+          <t>12[토지]경기도파주시파평면마산리</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>고양지욱</t>
+          <t>브</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>파주등기소</t>
+          <t>의정부지방범원</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>13[토지]경기도파주시파평면마산리</t>
+          <t>고양지욱</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>의정부지방</t>
+          <t>파주등기소</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>고양지원</t>
+          <t>13[토지]경기도파주시파평면마산리</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>파주능기소</t>
+          <t>의정부지방</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>훠기타사항</t>
+          <t>고양지원</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>일련번호부동산에관한권리의표처 SAW Sse</t>
+          <t>파주능기소</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>근 UW “Tou L ‘O 0 We</t>
+          <t>훠기타사항</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>래 CD 생성원인</t>
+          <t>일련번호부동산에관한권리의표처 SAW Sse</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>1 。 | (24)경기도파주시파평면마산리 | 의정부지방법원 _ | 62034년02월14일</t>
+          <t>근 UW “Tou L ‘O 0 We</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>113-38고양지원제10279호</t>
+          <t>래 CD 생성원인</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2 | [토지]경기도파주시파평면마산리 | 의정부지방법원102024년02월14일</t>
+          <t>1 。 | (24)경기도파주시파평면마산리 | 의정부지방법원 _ | 62034년02월14일</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>113-2고양지원제10279호</t>
+          <t>113-38고양지원제10279호</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>3 | [24]경기도파주시파평면마산리 | geal 102034년02월14일</t>
+          <t>2 | [토지]경기도파주시파평면마산리 | 의정부지방법원102024년02월14일</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>113-1고양지원제10279호</t>
+          <t>113-2고양지원제10279호</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>4 | [24]경기도파주시파평면마산리 | 의정부지방법원102034년02월14일</t>
+          <t>3 | [24]경기도파주시파평면마산리 | geal 102034년02월14일</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>산44-16고양지원제10279호</t>
+          <t>113-1고양지원제10279호</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>일련번호부동산에관한권리의표시관할능기소명순위번호</t>
+          <t>4 | [24]경기도파주시파평면마산리 | 의정부지방법원102034년02월14일</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>9[토지]경기도파주시파평면마산리 | ， 의정부지방법원2024년02월14일</t>
+          <t>산44-16고양지원제10279호</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>113-4고양지원제10279호</t>
+          <t>일련번호부동산에관한권리의표시관할능기소명순위번호</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>파주능기소설정계약으로</t>
+          <t>9[토지]경기도파주시파평면마산리 | ， 의정부지방법원2024년02월14일</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>파주시파평면마산리 ， 의정부지방법원2024년02월14일</t>
+          <t>113-4고양지원제10279호</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>고양지원제10279호</t>
+          <t>파주능기소설정계약으로</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>7 | [EAI]경기도파주시파평면마산리 | 의정부지방범원2024년02월14일</t>
+          <t>파주시파평면마산리 ， 의정부지방법원2024년02월14일</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>115-22고양지원제10279호</t>
+          <t>고양지원제10279호</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>8 . | [토지]경기도과주시파평면 abe 의정부치망밖원2024년02월14일</t>
+          <t>7 | [EAI]경기도파주시파평면마산리 | 의정부지방범원2024년02월14일</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>115-24고양착원제10279호</t>
+          <t>115-22고양지원제10279호</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>classed 설정계약으로</t>
+          <t>8 . | [토지]경기도과주시파평면 abe 의정부치망밖원2024년02월14일</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>9 | [토지]경기도파주시파평면마산리 | 의정부지방범원2024년02월14일</t>
+          <t>115-24고양착원제10279호</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>115-20고양지원제10279호</t>
+          <t>classed 설정계약으로</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>10 。 | [AI]경기도파주시파평먼마산리 | 의정부지방범원2024년02월14일</t>
+          <t>9 | [토지]경기도파주시파평면마산리 | 의정부지방범원2024년02월14일</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>115-23고양지원제10279호</t>
+          <t>115-20고양지원제10279호</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>11 | (4)경기도파주시파평먼마산리 | 의정부지방범원2024년02월14일</t>
+          <t>10 。 | [AI]경기도파주시파평먼마산리 | 의정부지방범원2024년02월14일</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>108-3고양지원제10279호</t>
+          <t>115-23고양지원제10279호</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>12 | [토지]경기도파주시파평면마산리 | 의정부지방법원 _ | 22024년02월14일</t>
+          <t>11 | (4)경기도파주시파평먼마산리 | 의정부지방범원2024년02월14일</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>108-4고양지원제10279호</t>
+          <t>108-3고양지원제10279호</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>일련번호부농산에관한권리의표시관할능기소명</t>
+          <t>12 | [토지]경기도파주시파평면마산리 | 의정부지방법원 _ | 22024년02월14일</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>[토지]경기도파주시파평면마산리 ， 의정부지방법원2024년02월14일</t>
+          <t>108-4고양지원제10279호</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>109-3고양지원제10279호</t>
+          <t>일련번호부농산에관한권리의표시관할능기소명</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>14[토지]경기도파주시파평면마산리 ， 의정부지방법원2024년02월14일</t>
+          <t>[토지]경기도파주시파평면마산리 ， 의정부지방법원2024년02월14일</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>116-15고양지원제10279호</t>
+          <t>109-3고양지원제10279호</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>ESS | 2024-558</t>
+          <t>14[토지]경기도파주시파평면마산리 ， 의정부지방법원2024년02월14일</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>[토지]경기도2024년04월04일</t>
+          <t>116-15고양지원제10279호</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>113-1원제29644호</t>
+          <t>ESS | 2024-558</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>[토지]경기도엉2024년04월04일</t>
+          <t>[토지]경기도2024년04월04일</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>113-2고양지원제29644호</t>
+          <t>113-1원제29644호</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>[토지]경기도파주시파평면마산리 ， 의정부지방법원2024년04월04일</t>
+          <t>[토지]경기도엉2024년04월04일</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>113-3고양지원제29644호</t>
+          <t>113-2고양지원제29644호</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>113-4고양지원제29644호</t>
+          <t>[토지]경기도파주시파평면마산리 ， 의정부지방법원2024년04월04일</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>생성원인변</t>
+          <t>113-3고양지원제29644호</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>9[토지]경기도파주시파평면마산리 ， 의정부지2024년04월04일</t>
+          <t>113-4고양지원제29644호</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>산44-16 ALA]¢ 제29644호</t>
+          <t>생성원인변</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>파주등설정계약으로</t>
+          <t>9[토지]경기도파주시파평면마산리 ， 의정부지2024년04월04일</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>6[토지]경기도파주시파평면마산리 ， 의정부지2024년04월04일</t>
+          <t>산44-16 ALA]¢ 제29644호</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>115-20고양지원제29644호</t>
+          <t>파주등설정계약으로</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>경기도파주시파평면마산리</t>
+          <t>6[토지]경기도파주시파평면마산리 ， 의정부지2024년04월04일</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>의정부지방법</t>
+          <t>115-20고양지원제29644호</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>의정부지</t>
+          <t>경기도파주시파평면마산리</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>파주능기</t>
+          <t>의정부지방법</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>파주등기</t>
+          <t>의정부지</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>11[토지]경기도파주시파평면마산리 ， 의정부지2024년04월04일</t>
+          <t>파주능기</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>108-3고양지원제29644호</t>
+          <t>파주등기</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>12[토지]경기도파주시파평면마산리 ， 의정부지방법2024년04월04일</t>
+          <t>11[토지]경기도파주시파평면마산리 ， 의정부지2024년04월04일</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>108-4고양지원제29644호</t>
+          <t>108-3고양지원제29644호</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>일련번호부동산에관한권리의표시관할등기소명순위번호</t>
+          <t>12[토지]경기도파주시파평면마산리 ， 의정부지방법2024년04월04일</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>13[토지]경기도파주시파평면마산리 ， 의정부지방법원42024년04월04일</t>
+          <t>108-4고양지원제29644호</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>109-3고양지원제39644호</t>
+          <t>일련번호부동산에관한권리의표시관할등기소명순위번호</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>[토지]경기도파주시파평면마산리2024년04월04일</t>
+          <t>13[토지]경기도파주시파평면마산리 ， 의정부지방법원42024년04월04일</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>116-15고양지원제39644호</t>
+          <t>109-3고양지원제39644호</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>기도파주시파평면마산리 | ， 의정부지2024년04월04일</t>
+          <t>[토지]경기도파주시파평면마산리2024년04월04일</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>산44-7고양지원제39644호</t>
+          <t>116-15고양지원제39644호</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>지원파주능기소</t>
+          <t>기도파주시파평면마산리 | ， 의정부지2024년04월04일</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>* 실선으로그어진부분은말소사항을표시함 * 기록사항없는갑구 , 을구는 ' 기록사항없음 ' 으로표시함 .</t>
+          <t>산44-7고양지원제39644호</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>* 증명서는컬러또는흑백으로출력가능함 .</t>
+          <t>지원파주능기소</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>* 본능기사항중명서는열람용이므로출력하신능기사항중명서는법적인효력이없습니다 .</t>
+          <t>* 실선으로그어진부분은말소사항을표시함 * 기록사항없는갑구 , 을구는 ' 기록사항없음 ' 으로표시함 .</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>주요등기사항요약(참고용)</t>
+          <t>* 증명서는컬러또는흑백으로출력가능함 .</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>떠 Ho</t>
+          <t>* 본능기사항중명서는열람용이므로출력하신능기사항중명서는법적인효력이없습니다 .</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>래누</t>
+          <t>주요등기사항요약(참고용)</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>태하</t>
+          <t>떠 Ho</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>ae: 홀</t>
+          <t>래누</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>10디 oO</t>
+          <t>태하</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>~ pm 발</t>
+          <t>ae: 홀</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>대 q]문매숙</t>
+          <t>10디 oO</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>~ jou jou . 그 ol!</t>
+          <t>~ pm 발</t>
         </is>
       </c>
     </row>
     <row r="244">
-      <c r="A244">
-        <f>» nd ad | aM 급 \</f>
-        <v/>
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>대 q]문매숙</t>
+        </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>110 一 야2비 ㅜ ob aril</t>
+          <t>~ jou jou . 그 ol!</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>ou o Ho | Sito oF 근 x ~</t>
+          <t>'=» nd ad | aM 급 \</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>겪 x Se | Spm S ee . 가</t>
+          <t>110 一 야2비 ㅜ ob aril</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>ㅇ ^ ~ 으 《 Ke 규</t>
+          <t>ou o Ho | Sito oF 근 x ~</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>3 ” | 음어애 et 으며는 .</t>
+          <t>겪 x Se | Spm S ee . 가</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>다사、」 S4 © io = jo”</t>
+          <t>ㅇ ^ ~ 으 《 Ke 규</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>中 묵 nh dH NE ONE “和 叫 olf! pr</t>
+          <t>3 ” | 음어애 et 으며는 .</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>ac Sg | Sa 퍼 | ow a x</t>
+          <t>다사、」 S4 © io = jo”</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>여돈 &lt; Moar | rear ° OK</t>
+          <t>中 묵 nh dH NE ONE “和 叫 olf! pr</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>꼬12 、 고으</t>
+          <t>ac Sg | Sa 퍼 | ow a x</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>jo , a 습농 oO</t>
+          <t>여돈 &lt; Moar | rear ° OK</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>ar 스 aK | OK arc + il 家 ay</t>
+          <t>꼬12 、 고으</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>NS ' 녀 | 디 ana 죠패 oy 로</t>
+          <t>jo , a 습농 oO</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>of ‘od 르넥당 NG TO 810 on 人 之</t>
+          <t>ar 스 aK | OK arc + il 家 ay</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>× 는2 全 x m PI! = ‘Oy ww</t>
+          <t>NS ' 녀 | 디 ana 죠패 oy 로</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>oy 部 응 \ 0 * eae</t>
+          <t>of ‘od 르넥당 NG TO 810 on 人 之</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>of oF 패 nu 0 nye | 9 中 5 中</t>
+          <t>× 는2 全 x m PI! = ‘Oy ww</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>人 0 K Ft! 6 = 리 = Ho 동 yo 때</t>
+          <t>oy 部 응 \ 0 * eae</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>KX p Mo ~ 디없 a io | 이 | 8예</t>
+          <t>of oF 패 nu 0 nye | 9 中 5 中</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>當 Be 2 .에0껄8 No | ㅇ 02끓뺀인 . of)a</t>
+          <t>人 0 K Ft! 6 = 리 = Ho 동 yo 때</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>써 Me = ral oS mS | S | me 에픈패문</t>
+          <t>KX p Mo ~ 디없 a io | 이 | 8예</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>패 “ 럼운국의 | 해으 | 클이눈우제우</t>
+          <t>當 Be 2 .에0껄8 No | ㅇ 02끓뺀인 . of)a</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>__ 뭐구스구 NK ~ 스눈 No N 더 x ah 비</t>
+          <t>써 Me = ral oS mS | S | me 에픈패문</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>조 eal Hol i RX | RK | aE oF 는의께</t>
+          <t>패 “ 럼운국의 | 해으 | 클이눈우제우</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>wm nr 계90짜 ob</t>
+          <t>__ 뭐구스구 NK ~ 스눈 No N 더 x ah 비</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>x lo 깝 xo ~ Ko dd Fe</t>
+          <t>조 eal Hol i RX | RK | aE oF 는의께</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>10스 Fe x Ke</t>
+          <t>wm nr 계90짜 ob</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>그 ~ | 스 of 字 ulo ob 이이</t>
+          <t>x lo 깝 xo ~ Ko dd Fe</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>2 一 NE x 깥패는 , 3</t>
+          <t>10스 Fe x Ke</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>ag 에이는 ew RIS | &amp; Code</t>
+          <t>그 ~ | 스 of 字 ulo ob 이이</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>ㅇ w 급 &gt; 70 &lt; 능</t>
+          <t>2 一 NE x 깥패는 , 3</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>全 密 너0히 BK o NO FO</t>
+          <t>ag 에이는 ew RIS | &amp; Code</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>트도 ㅡ 000 | 9이 vaya blo TF</t>
+          <t>ㅇ w 급 &gt; 70 &lt; 능</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>blo X ~ ooh)oO 빌 \ &lt; 스</t>
+          <t>全 密 너0히 BK o NO FO</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>He} oe ele | o | 준께 —e ane</t>
+          <t>트도 ㅡ 000 | 9이 vaya blo TF</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>KE 레 一 說 i mm joo THT 때 Me op</t>
+          <t>blo X ~ ooh)oO 빌 \ &lt; 스</t>
         </is>
       </c>
     </row>
     <row r="281">
-      <c r="A281">
-        <f> = | ue ㄷ . RYO 선</f>
-        <v/>
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>He} oe ele | o | 준께 —e ane</t>
+        </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>쩌)3 my 써1 ~ No ak! &lt;0</t>
+          <t>KE 레 一 說 i mm joo THT 때 Me op</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>그음 . ~ rule me KF</t>
+          <t>'= = | ue ㄷ . RYO 선</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>: 202643월319오후5시25분59초</t>
+          <t>쩌)3 my 써1 ~ No ak! &lt;0</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
+        <is>
+          <t>그음 . ~ rule me KF</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>: 202643월319오후5시25분59초</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
         <is>
           <t>출력일시</t>
         </is>

</xml_diff>